<commit_message>
docs: enrich SDLC excel workbooks with data validation, team guides, and massive example data
</commit_message>
<xml_diff>
--- a/reference/governance/sdlc/assets/evolith-new-system-tracking-workbook.xlsx
+++ b/reference/governance/sdlc/assets/evolith-new-system-tracking-workbook.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contexto del Sistema" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa vs UMS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro de Decisiones (ADRs)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDLC Tracker" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-Instrucciones Operativas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02-Ficha Técnica" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-Mapeo vs UMS (Reuso)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-Tracker de ADRs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05-Entregables SDLC (Scorecard)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +45,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001E3A5F"/>
         <bgColor rgb="001E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+        <bgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,10 +78,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,48 +454,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Propiedad</t>
+          <t>Ceremonia Ágil</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Detalle Registrado</t>
+          <t>Actividad a realizar en este Workbook</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Participantes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Nombre del Sistema</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sprint Planning</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Revisar la pestaña '05-Entregables SDLC' para verificar si faltan artefactos de diseño antes de codificar.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>PO, Tech Lead</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Repositorio GitHub</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Arquitectura (Sync)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Actualizar el '04-Tracker de ADRs' si se tomó una decisión sobre base de datos, colas, o infraestructura.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Arquitecto, TL</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Justificación de Negocio</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sprint Review</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Revisar los módulos completados contra la '03-Mapeo vs UMS' para ver avance real.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -489,122 +541,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="49" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Módulo / Funcionalidad</t>
+          <t>Propiedad Arquitectónica</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>¿Reusar patrón UMS?</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>¿Adaptar patrón UMS?</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>¿Desarrollo Nuevo?</t>
+          <t>Detalle de Implementación</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Autenticación</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>[ ]</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Nombre Oficial del Sistema</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Sistema Core de Tarjetas (Ejemplo)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Manejo de Permisos Corporativos</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>[ ]</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Código de Proyecto / Centro de Costos</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>PRJ-99901</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Auditoría y Trazas</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>[ ]</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Clasificación de Criticidad (Tier)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 - Mission Critical</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Lógica Core Especializada</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>[ ]</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>RTO (Recovery Time Objective)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Menor a 4 horas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>RPO (Recovery Point Objective)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Menor a 5 minutos</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Repositorio Git (Backend)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/empresa/core-tarjetas-api</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Repositorio Git (Frontend)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/empresa/core-tarjetas-web</t>
         </is>
       </c>
     </row>
@@ -619,59 +655,156 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Módulo / Bounded Context</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Título de la Decisión</t>
+          <t>¿Estrategia?</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Estatus (Draft/Accepted)</t>
+          <t>Justificación / Detalle Técnico</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Impacto</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>URL Evidencia</t>
+          <t>Estatus</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ADR-0001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Topología Base</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Autenticación OIDC (Keycloak)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Reusar UMS</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Se utilizará el Auth Server institucional idéntico a UMS.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Listo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Usuarios Admin</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Adaptar UMS</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Se extenderá el schema de UMS para incluir 'Tipo de Tarjeta'.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>En Desarrollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Motor de Originación Crediticia</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo Desarrollo</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Lógica core de negocio propia del banco.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>En Desarrollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Motor de Reglas Antifraude</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Software Comercial (COTS)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Integración vía API REST con proveedor externo.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Notificaciones SMS/Email</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Adaptar UMS</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Se reutilizará el dispatcher de UMS agregando AWS SNS.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="D2 D3 D4 D5 D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pendiente,En Desarrollo,Listo,Cancelado"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2 B3 B4 B5 B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Reusar UMS,Adaptar UMS,Nuevo Desarrollo,Software Comercial (COTS)"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -682,136 +815,529 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Fase</t>
+          <t>ID Decisión</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Título Breve</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Estatus (ADR)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Descripción del Impacto</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>URL Confluence/GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ADR-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Base de Datos para Transacciones</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Se elige PostgreSQL sobre MongoDB por consistencia ACID estricta en pagos.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://link-al-adr.com/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ADR-0002</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Manejo de Eventos Asíncronos</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Uso de Kafka para notificar al core cuando la originación se apruebe.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>https://link-al-adr.com/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ADR-0003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Framework UI Frontend</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Uso de React 18 alineado a los blueprints base de Evolith.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://link-al-adr.com/3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2 C3 C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Draft,Proposed,Accepted,Rejected,Deprecated"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fase SDLC</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Artefacto</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Obligatoriedad</t>
+          <t>Nivel de Obligatoriedad</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Estatus (Pendiente/Done)</t>
+          <t>Estatus del Entregable</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>URL del Documento</t>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>URL Evidencia</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>1. Concepción</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>PRD Aprobado</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Obligatorio</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Product Requirements Document (PRD)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>PO</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>http://confluence/prd</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>1. Concepción</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Aprobación Presupuestal / Charter</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2. Diseño</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ADRs Mínimos Publicados</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Obligatorio</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Modelo Entidad Relación (MER)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Arquitecto</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2. Diseño</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Diagramas de Secuencia APIs</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>En Redacción</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Tech Lead</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2. Diseño</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Diseño de Interfaz UX/UI (Figma)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Condicional</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>3. Construcción</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Contratos API Swagger/OpenAPI</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>En Redacción</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Desarrollador</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>3. Construcción</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Reporte Cobertura SonarQube (&gt;80%)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>4. Validación</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Test Summary Report Limpio</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Obligatorio</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Reporte Análisis Estático SAST</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>SecOps</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>4. Validación</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Reporte de Pruebas UAT Firmado</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>4. Validación</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Performance Test Summary</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Condicional</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Arquitecto</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>5. Entrega</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Release Notes Generadas</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Obligatorio</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>[ ]</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Release Notes &amp; Changelog</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Tech Lead</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>5. Entrega</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Aprobación Comité de Pases (CAB)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Mandatorio</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2 D3 D4 D5 D6 D7 D8 D9 D10 D11 D12 D13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pendiente,En Redacción,Bloqueado,Aprobado,No Aplica"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: generalize new system tracking workbook, removing UMS dependencies
</commit_message>
<xml_diff>
--- a/reference/governance/sdlc/assets/evolith-new-system-tracking-workbook.xlsx
+++ b/reference/governance/sdlc/assets/evolith-new-system-tracking-workbook.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-Instrucciones Operativas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02-Ficha Técnica" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-Mapeo vs UMS (Reuso)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-Definición de Módulos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-Tracker de ADRs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05-Entregables SDLC (Scorecard)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
@@ -521,7 +521,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Revisar los módulos completados contra la '03-Mapeo vs UMS' para ver avance real.</t>
+          <t>Revisar la pestaña de '03-Definición de Módulos' para reflejar el progreso de los Bounded Contexts.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -545,7 +545,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="49" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -568,7 +568,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Sistema Core de Tarjetas (Ejemplo)</t>
+          <t>Sistema Core de Negocio (Ejemplo)</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/empresa/core-tarjetas-api</t>
+          <t>https://github.com/empresa/mi-sistema-api</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/empresa/core-tarjetas-web</t>
+          <t>https://github.com/empresa/mi-sistema-web</t>
         </is>
       </c>
     </row>
@@ -655,13 +655,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -672,7 +672,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>¿Estrategia?</t>
+          <t>¿Estrategia de Arquitectura?</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -682,46 +682,46 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Estatus</t>
+          <t>Estatus de Construcción</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Autenticación OIDC (Keycloak)</t>
+          <t>Gestión de Clientes (CRM)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Reusar UMS</t>
+          <t>Software COTS</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Se utilizará el Auth Server institucional idéntico a UMS.</t>
+          <t>Integración con Salesforce vía APIs. No se desarrollará lógica custom.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Listo</t>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Usuarios Admin</t>
+          <t>Motor de Facturación</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Adaptar UMS</t>
+          <t>Desarrollo In-House</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Se extenderá el schema de UMS para incluir 'Tipo de Tarjeta'.</t>
+          <t>Lógica core de negocio altamente personalizada.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -733,64 +733,42 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Motor de Originación Crediticia</t>
+          <t>Módulo de Autenticación</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Nuevo Desarrollo</t>
+          <t>Patrón Evolith Estándar</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Lógica core de negocio propia del banco.</t>
+          <t>Se adopta el blueprint estándar corporativo basado en OIDC.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>En Desarrollo</t>
+          <t>Listo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Motor de Reglas Antifraude</t>
+          <t>Pasarela de Pagos</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Software Comercial (COTS)</t>
+          <t>Servicio SaaS Externo</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Integración vía API REST con proveedor externo.</t>
+          <t>Integración con Stripe usando el SDK oficial.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Notificaciones SMS/Email</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Adaptar UMS</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Se reutilizará el dispatcher de UMS agregando AWS SNS.</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -798,11 +776,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="D2 D3 D4 D5 D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2 D3 D4 D5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,En Desarrollo,Listo,Cancelado"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2 B3 B4 B5 B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Reusar UMS,Adaptar UMS,Nuevo Desarrollo,Software Comercial (COTS)"</formula1>
+    <dataValidation sqref="B2 B3 B4 B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Desarrollo In-House,Patrón Evolith Estándar,Software COTS,Servicio SaaS Externo"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>